<commit_message>
Update MLB weather 2026-08-17 05:02 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v5_2026_08_17.xlsx
+++ b/mlb_weather_professional_v5_2026_08_17.xlsx
@@ -443,10 +443,10 @@
     <t>Density 75 | Wind 59 | Temp 57 | Altitude 65 | Confidence 87%</t>
   </si>
   <si>
-    <t>Density 72 | Wind 49 | Temp 61 | Altitude 62 | Confidence 89%</t>
-  </si>
-  <si>
-    <t>Density 77 | Wind 56 | Temp 55 | Altitude 66 | Confidence 91%</t>
+    <t>Density 72 | Wind 49 | Temp 61 | Altitude 62 | Confidence 87%</t>
+  </si>
+  <si>
+    <t>Density 77 | Wind 56 | Temp 55 | Altitude 66 | Confidence 90%</t>
   </si>
   <si>
     <t>Density 64 | Wind 47 | Temp 51 | Altitude 57 | Confidence 93%</t>
@@ -488,9 +488,6 @@
     <t>STEADY</t>
   </si>
   <si>
-    <t>WORSENING</t>
-  </si>
-  <si>
     <t>WORSENING RAPIDLY</t>
   </si>
   <si>
@@ -500,43 +497,46 @@
     <t>NONE (ROOF)</t>
   </si>
   <si>
+    <t>ELEVATED</t>
+  </si>
+  <si>
     <t>LOW</t>
   </si>
   <si>
     <t>MEDIUM</t>
   </si>
   <si>
-    <t>2026-08-17 04:59:25 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-08-17 04:59:27 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-08-17 04:59:28 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-08-17 04:59:30 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-08-17 04:59:31 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-08-17 04:59:32 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-08-17 04:59:33 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-08-17 04:59:34 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-08-17 04:59:36 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-08-17 04:59:37 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-08-17 04:59:38 PM PDT</t>
+    <t>2026-08-17 05:01:03 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-08-17 05:01:11 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-08-17 05:01:19 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-08-17 05:01:26 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-08-17 05:01:34 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-08-17 05:01:41 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-08-17 05:01:48 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-08-17 05:01:54 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-08-17 05:01:59 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-08-17 05:02:04 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-08-17 05:02:09 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -899,37 +899,37 @@
     <t>09:40 PM MDT</t>
   </si>
   <si>
-    <t>2026-08-17 23:59:25 UTC</t>
-  </si>
-  <si>
-    <t>2026-08-17 23:59:27 UTC</t>
-  </si>
-  <si>
-    <t>2026-08-17 23:59:28 UTC</t>
-  </si>
-  <si>
-    <t>2026-08-17 23:59:30 UTC</t>
-  </si>
-  <si>
-    <t>2026-08-17 23:59:31 UTC</t>
-  </si>
-  <si>
-    <t>2026-08-17 23:59:32 UTC</t>
-  </si>
-  <si>
-    <t>2026-08-17 23:59:33 UTC</t>
-  </si>
-  <si>
-    <t>2026-08-17 23:59:34 UTC</t>
-  </si>
-  <si>
-    <t>2026-08-17 23:59:36 UTC</t>
-  </si>
-  <si>
-    <t>2026-08-17 23:59:37 UTC</t>
-  </si>
-  <si>
-    <t>2026-08-17 23:59:38 UTC</t>
+    <t>2026-08-18 00:01:03 UTC</t>
+  </si>
+  <si>
+    <t>2026-08-18 00:01:11 UTC</t>
+  </si>
+  <si>
+    <t>2026-08-18 00:01:19 UTC</t>
+  </si>
+  <si>
+    <t>2026-08-18 00:01:26 UTC</t>
+  </si>
+  <si>
+    <t>2026-08-18 00:01:34 UTC</t>
+  </si>
+  <si>
+    <t>2026-08-18 00:01:41 UTC</t>
+  </si>
+  <si>
+    <t>2026-08-18 00:01:48 UTC</t>
+  </si>
+  <si>
+    <t>2026-08-18 00:01:54 UTC</t>
+  </si>
+  <si>
+    <t>2026-08-18 00:01:59 UTC</t>
+  </si>
+  <si>
+    <t>2026-08-18 00:02:04 UTC</t>
+  </si>
+  <si>
+    <t>2026-08-18 00:02:09 UTC</t>
   </si>
   <si>
     <t>2026-08-17T22:34:52+00:00</t>
@@ -1862,7 +1862,7 @@
         <v>16</v>
       </c>
       <c r="AU2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="AV2">
         <v>28.2</v>
@@ -1877,7 +1877,7 @@
         <v>161</v>
       </c>
       <c r="AZ2">
-        <v>84.59999999999999</v>
+        <v>86.2</v>
       </c>
       <c r="BA2">
         <v>5</v>
@@ -1945,7 +1945,7 @@
         <v>133</v>
       </c>
       <c r="V3">
-        <v>2.7</v>
+        <v>2.4</v>
       </c>
       <c r="W3">
         <v>50</v>
@@ -2020,7 +2020,7 @@
         <v>15</v>
       </c>
       <c r="AU3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="AV3">
         <v>0</v>
@@ -2035,7 +2035,7 @@
         <v>162</v>
       </c>
       <c r="AZ3">
-        <v>262.2</v>
+        <v>264</v>
       </c>
       <c r="BA3">
         <v>5</v>
@@ -2103,7 +2103,7 @@
         <v>133</v>
       </c>
       <c r="V4">
-        <v>29.9</v>
+        <v>28.1</v>
       </c>
       <c r="W4">
         <v>62.2</v>
@@ -2124,7 +2124,7 @@
         <v>3.7</v>
       </c>
       <c r="AC4">
-        <v>87.3</v>
+        <v>87</v>
       </c>
       <c r="AD4" t="s">
         <v>148</v>
@@ -2169,7 +2169,7 @@
         <v>153</v>
       </c>
       <c r="AR4">
-        <v>4.6</v>
+        <v>4.7</v>
       </c>
       <c r="AS4">
         <v>-0.32</v>
@@ -2178,10 +2178,10 @@
         <v>16</v>
       </c>
       <c r="AU4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="AV4">
-        <v>28</v>
+        <v>26.1</v>
       </c>
       <c r="AW4" t="s">
         <v>159</v>
@@ -2193,7 +2193,7 @@
         <v>163</v>
       </c>
       <c r="AZ4">
-        <v>84.59999999999999</v>
+        <v>86.5</v>
       </c>
       <c r="BA4">
         <v>5</v>
@@ -2261,10 +2261,10 @@
         <v>133</v>
       </c>
       <c r="V5">
-        <v>18.9</v>
+        <v>18</v>
       </c>
       <c r="W5">
-        <v>57.4</v>
+        <v>57.3</v>
       </c>
       <c r="X5" t="s">
         <v>136</v>
@@ -2282,7 +2282,7 @@
         <v>2.2</v>
       </c>
       <c r="AC5">
-        <v>89</v>
+        <v>87.2</v>
       </c>
       <c r="AD5" t="s">
         <v>150</v>
@@ -2327,7 +2327,7 @@
         <v>154</v>
       </c>
       <c r="AR5">
-        <v>0.8</v>
+        <v>-0.7</v>
       </c>
       <c r="AS5">
         <v>-0.02</v>
@@ -2336,22 +2336,22 @@
         <v>17</v>
       </c>
       <c r="AU5" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="AV5">
-        <v>44.1</v>
+        <v>47.1</v>
       </c>
       <c r="AW5" t="s">
         <v>159</v>
       </c>
       <c r="AX5">
-        <v>6.9</v>
+        <v>11.1</v>
       </c>
       <c r="AY5" t="s">
         <v>164</v>
       </c>
       <c r="AZ5">
-        <v>230.6</v>
+        <v>232.5</v>
       </c>
       <c r="BA5">
         <v>5</v>
@@ -2419,7 +2419,7 @@
         <v>133</v>
       </c>
       <c r="V6">
-        <v>21.2</v>
+        <v>18.2</v>
       </c>
       <c r="W6">
         <v>61.2</v>
@@ -2437,10 +2437,10 @@
         <v>5</v>
       </c>
       <c r="AB6">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="AC6">
-        <v>90.59999999999999</v>
+        <v>90.2</v>
       </c>
       <c r="AD6" t="s">
         <v>148</v>
@@ -2485,7 +2485,7 @@
         <v>152</v>
       </c>
       <c r="AR6">
-        <v>2.1</v>
+        <v>2</v>
       </c>
       <c r="AS6">
         <v>-0.73</v>
@@ -2497,7 +2497,7 @@
         <v>159</v>
       </c>
       <c r="AV6">
-        <v>18.6</v>
+        <v>17</v>
       </c>
       <c r="AW6" t="s">
         <v>159</v>
@@ -2509,7 +2509,7 @@
         <v>165</v>
       </c>
       <c r="AZ6">
-        <v>72.7</v>
+        <v>74.7</v>
       </c>
       <c r="BA6">
         <v>5</v>
@@ -2598,7 +2598,7 @@
         <v>0.8</v>
       </c>
       <c r="AC7">
-        <v>93</v>
+        <v>93.2</v>
       </c>
       <c r="AD7" t="s">
         <v>150</v>
@@ -2640,10 +2640,10 @@
         <v>88.3</v>
       </c>
       <c r="AQ7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="AR7">
-        <v>-2.2</v>
+        <v>-1.3</v>
       </c>
       <c r="AS7">
         <v>-0.36</v>
@@ -2667,7 +2667,7 @@
         <v>166</v>
       </c>
       <c r="AZ7">
-        <v>370.2</v>
+        <v>372.4</v>
       </c>
       <c r="BA7">
         <v>5</v>
@@ -2756,7 +2756,7 @@
         <v>0.5</v>
       </c>
       <c r="AC8">
-        <v>90.40000000000001</v>
+        <v>90.2</v>
       </c>
       <c r="AD8" t="s">
         <v>150</v>
@@ -2798,10 +2798,10 @@
         <v>81.8</v>
       </c>
       <c r="AQ8" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="AR8">
-        <v>-5.5</v>
+        <v>-5.7</v>
       </c>
       <c r="AS8">
         <v>-0.3</v>
@@ -2819,13 +2819,13 @@
         <v>159</v>
       </c>
       <c r="AX8">
-        <v>16.3</v>
+        <v>16.2</v>
       </c>
       <c r="AY8" t="s">
         <v>167</v>
       </c>
       <c r="AZ8">
-        <v>195.3</v>
+        <v>197.5</v>
       </c>
       <c r="BA8">
         <v>5</v>
@@ -2959,7 +2959,7 @@
         <v>155</v>
       </c>
       <c r="AR9">
-        <v>-3.3</v>
+        <v>-4.4</v>
       </c>
       <c r="AS9">
         <v>-0.18</v>
@@ -2983,7 +2983,7 @@
         <v>168</v>
       </c>
       <c r="AZ9">
-        <v>332.7</v>
+        <v>335</v>
       </c>
       <c r="BA9">
         <v>5</v>
@@ -3051,7 +3051,7 @@
         <v>133</v>
       </c>
       <c r="V10">
-        <v>5.6</v>
+        <v>8</v>
       </c>
       <c r="W10">
         <v>63.2</v>
@@ -3069,10 +3069,10 @@
         <v>6</v>
       </c>
       <c r="AB10">
-        <v>4</v>
+        <v>3.9</v>
       </c>
       <c r="AC10">
-        <v>92.3</v>
+        <v>91.7</v>
       </c>
       <c r="AD10" t="s">
         <v>148</v>
@@ -3117,7 +3117,7 @@
         <v>152</v>
       </c>
       <c r="AR10">
-        <v>3.9</v>
+        <v>3.7</v>
       </c>
       <c r="AS10">
         <v>-0.9</v>
@@ -3141,7 +3141,7 @@
         <v>169</v>
       </c>
       <c r="AZ10">
-        <v>92.5</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="BA10">
         <v>5</v>
@@ -3272,10 +3272,10 @@
         <v>71.59999999999999</v>
       </c>
       <c r="AQ11" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="AR11">
-        <v>0.3</v>
+        <v>1.7</v>
       </c>
       <c r="AS11">
         <v>0.59</v>
@@ -3299,7 +3299,7 @@
         <v>170</v>
       </c>
       <c r="AZ11">
-        <v>253.5</v>
+        <v>256</v>
       </c>
       <c r="BA11">
         <v>5</v>
@@ -3433,7 +3433,7 @@
         <v>153</v>
       </c>
       <c r="AR12">
-        <v>7.4</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="AS12">
         <v>0.57</v>
@@ -3457,7 +3457,7 @@
         <v>171</v>
       </c>
       <c r="AZ12">
-        <v>313.4</v>
+        <v>315.9</v>
       </c>
       <c r="BA12">
         <v>5</v>
@@ -3927,7 +3927,7 @@
         <v>303</v>
       </c>
       <c r="J2">
-        <v>84.59999999999999</v>
+        <v>86.2</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -4191,7 +4191,7 @@
         <v>28.2</v>
       </c>
       <c r="CT2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="CU2">
         <v>15.9</v>
@@ -4241,7 +4241,7 @@
         <v>303</v>
       </c>
       <c r="J3">
-        <v>84.59999999999999</v>
+        <v>86.2</v>
       </c>
       <c r="K3">
         <v>0</v>
@@ -4505,7 +4505,7 @@
         <v>26.9</v>
       </c>
       <c r="CT3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="CU3">
         <v>18.1</v>
@@ -4555,7 +4555,7 @@
         <v>303</v>
       </c>
       <c r="J4">
-        <v>84.59999999999999</v>
+        <v>86.2</v>
       </c>
       <c r="K4">
         <v>0</v>
@@ -4819,7 +4819,7 @@
         <v>27.1</v>
       </c>
       <c r="CT4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="CU4">
         <v>18.9</v>
@@ -4869,7 +4869,7 @@
         <v>303</v>
       </c>
       <c r="J5">
-        <v>84.59999999999999</v>
+        <v>86.2</v>
       </c>
       <c r="K5">
         <v>0</v>
@@ -5133,7 +5133,7 @@
         <v>28</v>
       </c>
       <c r="CT5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="CU5">
         <v>16.3</v>
@@ -5183,7 +5183,7 @@
         <v>304</v>
       </c>
       <c r="J6">
-        <v>262.2</v>
+        <v>264</v>
       </c>
       <c r="K6">
         <v>0</v>
@@ -5198,7 +5198,7 @@
         <v>0.92</v>
       </c>
       <c r="O6">
-        <v>1.28</v>
+        <v>1.26</v>
       </c>
       <c r="P6">
         <v>5.3</v>
@@ -5270,7 +5270,7 @@
         <v>8</v>
       </c>
       <c r="AM6">
-        <v>2.7</v>
+        <v>2.4</v>
       </c>
       <c r="AN6">
         <v>0</v>
@@ -5447,7 +5447,7 @@
         <v>0</v>
       </c>
       <c r="CT6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="CU6">
         <v>3.3</v>
@@ -5497,7 +5497,7 @@
         <v>304</v>
       </c>
       <c r="J7">
-        <v>262.2</v>
+        <v>264</v>
       </c>
       <c r="K7">
         <v>0</v>
@@ -5512,7 +5512,7 @@
         <v>1.2</v>
       </c>
       <c r="O7">
-        <v>1.31</v>
+        <v>1.1</v>
       </c>
       <c r="P7">
         <v>10.5</v>
@@ -5539,10 +5539,10 @@
         <v>0.0833</v>
       </c>
       <c r="X7">
-        <v>6.1</v>
+        <v>6</v>
       </c>
       <c r="Y7">
-        <v>93.8</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="Z7">
         <v>53.2</v>
@@ -5761,7 +5761,7 @@
         <v>0</v>
       </c>
       <c r="CT7" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="CU7">
         <v>6.2</v>
@@ -5811,7 +5811,7 @@
         <v>304</v>
       </c>
       <c r="J8">
-        <v>262.2</v>
+        <v>264</v>
       </c>
       <c r="K8">
         <v>0.1</v>
@@ -5826,7 +5826,7 @@
         <v>2.2</v>
       </c>
       <c r="O8">
-        <v>1.5</v>
+        <v>1.22</v>
       </c>
       <c r="P8">
         <v>16.2</v>
@@ -5853,10 +5853,10 @@
         <v>0.0833</v>
       </c>
       <c r="X8">
-        <v>13.7</v>
+        <v>13.6</v>
       </c>
       <c r="Y8">
-        <v>91.59999999999999</v>
+        <v>91.7</v>
       </c>
       <c r="Z8">
         <v>53.1</v>
@@ -6075,7 +6075,7 @@
         <v>0</v>
       </c>
       <c r="CT8" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="CU8">
         <v>4</v>
@@ -6125,7 +6125,7 @@
         <v>304</v>
       </c>
       <c r="J9">
-        <v>262.2</v>
+        <v>264</v>
       </c>
       <c r="K9">
         <v>1.1</v>
@@ -6140,7 +6140,7 @@
         <v>2.05</v>
       </c>
       <c r="O9">
-        <v>1.5</v>
+        <v>1.22</v>
       </c>
       <c r="P9">
         <v>14.4</v>
@@ -6167,10 +6167,10 @@
         <v>0.0833</v>
       </c>
       <c r="X9">
-        <v>15.5</v>
+        <v>15.4</v>
       </c>
       <c r="Y9">
-        <v>91.09999999999999</v>
+        <v>91.2</v>
       </c>
       <c r="Z9">
         <v>53.1</v>
@@ -6212,7 +6212,7 @@
         <v>7.4</v>
       </c>
       <c r="AM9">
-        <v>0.9</v>
+        <v>0.4</v>
       </c>
       <c r="AN9">
         <v>0</v>
@@ -6389,7 +6389,7 @@
         <v>0</v>
       </c>
       <c r="CT9" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="CU9">
         <v>3.5</v>
@@ -6439,7 +6439,7 @@
         <v>303</v>
       </c>
       <c r="J10">
-        <v>84.59999999999999</v>
+        <v>86.5</v>
       </c>
       <c r="K10">
         <v>0</v>
@@ -6454,7 +6454,7 @@
         <v>0.77</v>
       </c>
       <c r="O10">
-        <v>29.14</v>
+        <v>30.45</v>
       </c>
       <c r="P10">
         <v>18.8</v>
@@ -6481,13 +6481,13 @@
         <v>0.6667</v>
       </c>
       <c r="X10">
-        <v>15.8</v>
+        <v>16.3</v>
       </c>
       <c r="Y10">
-        <v>84.8</v>
+        <v>84.59999999999999</v>
       </c>
       <c r="Z10">
-        <v>69.7</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="AA10">
         <v>1</v>
@@ -6526,7 +6526,7 @@
         <v>23.9</v>
       </c>
       <c r="AM10">
-        <v>29.9</v>
+        <v>28.1</v>
       </c>
       <c r="AN10">
         <v>0.001</v>
@@ -6700,10 +6700,10 @@
         <v>56.6</v>
       </c>
       <c r="CS10">
-        <v>26.9</v>
+        <v>25.9</v>
       </c>
       <c r="CT10" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="CU10">
         <v>14.6</v>
@@ -6753,7 +6753,7 @@
         <v>303</v>
       </c>
       <c r="J11">
-        <v>84.59999999999999</v>
+        <v>86.5</v>
       </c>
       <c r="K11">
         <v>0</v>
@@ -6768,7 +6768,7 @@
         <v>0.5</v>
       </c>
       <c r="O11">
-        <v>27.3</v>
+        <v>30.62</v>
       </c>
       <c r="P11">
         <v>10.6</v>
@@ -6795,13 +6795,13 @@
         <v>0.6667</v>
       </c>
       <c r="X11">
-        <v>15.9</v>
+        <v>17.1</v>
       </c>
       <c r="Y11">
-        <v>90.40000000000001</v>
+        <v>89.8</v>
       </c>
       <c r="Z11">
-        <v>69</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="AA11">
         <v>1</v>
@@ -6840,7 +6840,7 @@
         <v>53.1</v>
       </c>
       <c r="AM11">
-        <v>23.4</v>
+        <v>19.9</v>
       </c>
       <c r="AN11">
         <v>0.011</v>
@@ -7014,10 +7014,10 @@
         <v>58.9</v>
       </c>
       <c r="CS11">
-        <v>28</v>
+        <v>26.1</v>
       </c>
       <c r="CT11" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="CU11">
         <v>4.5</v>
@@ -7067,10 +7067,10 @@
         <v>303</v>
       </c>
       <c r="J12">
-        <v>84.59999999999999</v>
+        <v>86.5</v>
       </c>
       <c r="K12">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="L12">
         <v>5</v>
@@ -7082,7 +7082,7 @@
         <v>1.43</v>
       </c>
       <c r="O12">
-        <v>24.45</v>
+        <v>26.27</v>
       </c>
       <c r="P12">
         <v>13.1</v>
@@ -7109,10 +7109,10 @@
         <v>0.6667</v>
       </c>
       <c r="X12">
-        <v>19.2</v>
+        <v>19.8</v>
       </c>
       <c r="Y12">
-        <v>87.2</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="Z12">
         <v>61.9</v>
@@ -7154,7 +7154,7 @@
         <v>52.2</v>
       </c>
       <c r="AM12">
-        <v>17.3</v>
+        <v>15.2</v>
       </c>
       <c r="AN12">
         <v>0.006</v>
@@ -7328,7 +7328,7 @@
         <v>61.8</v>
       </c>
       <c r="CS12">
-        <v>19.6</v>
+        <v>18.5</v>
       </c>
       <c r="CT12" t="s">
         <v>159</v>
@@ -7381,10 +7381,10 @@
         <v>303</v>
       </c>
       <c r="J13">
-        <v>84.59999999999999</v>
+        <v>86.5</v>
       </c>
       <c r="K13">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="L13">
         <v>5</v>
@@ -7396,7 +7396,7 @@
         <v>1.57</v>
       </c>
       <c r="O13">
-        <v>15.94</v>
+        <v>16.27</v>
       </c>
       <c r="P13">
         <v>29.6</v>
@@ -7423,7 +7423,7 @@
         <v>0.6667</v>
       </c>
       <c r="X13">
-        <v>15.3</v>
+        <v>15.4</v>
       </c>
       <c r="Y13">
         <v>88</v>
@@ -7468,7 +7468,7 @@
         <v>62</v>
       </c>
       <c r="AM13">
-        <v>8.199999999999999</v>
+        <v>7.8</v>
       </c>
       <c r="AN13">
         <v>0</v>
@@ -7642,7 +7642,7 @@
         <v>63.2</v>
       </c>
       <c r="CS13">
-        <v>11</v>
+        <v>10.7</v>
       </c>
       <c r="CT13" t="s">
         <v>159</v>
@@ -7695,7 +7695,7 @@
         <v>305</v>
       </c>
       <c r="J14">
-        <v>230.6</v>
+        <v>232.5</v>
       </c>
       <c r="K14">
         <v>0</v>
@@ -7710,7 +7710,7 @@
         <v>1.2</v>
       </c>
       <c r="O14">
-        <v>21.28</v>
+        <v>22.3</v>
       </c>
       <c r="P14">
         <v>60</v>
@@ -7737,10 +7737,10 @@
         <v>0.6667</v>
       </c>
       <c r="X14">
-        <v>19.8</v>
+        <v>20.2</v>
       </c>
       <c r="Y14">
-        <v>87.3</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="Z14">
         <v>52.2</v>
@@ -7782,7 +7782,7 @@
         <v>44</v>
       </c>
       <c r="AM14">
-        <v>18.9</v>
+        <v>18</v>
       </c>
       <c r="AN14">
         <v>0.003</v>
@@ -7956,10 +7956,10 @@
         <v>50.8</v>
       </c>
       <c r="CS14">
-        <v>21.6</v>
+        <v>21.1</v>
       </c>
       <c r="CT14" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="CU14">
         <v>6.9</v>
@@ -8009,7 +8009,7 @@
         <v>305</v>
       </c>
       <c r="J15">
-        <v>230.6</v>
+        <v>232.5</v>
       </c>
       <c r="K15">
         <v>0</v>
@@ -8024,7 +8024,7 @@
         <v>0.82</v>
       </c>
       <c r="O15">
-        <v>25.79</v>
+        <v>22.05</v>
       </c>
       <c r="P15">
         <v>65.3</v>
@@ -8051,13 +8051,13 @@
         <v>0.6667</v>
       </c>
       <c r="X15">
-        <v>18.9</v>
+        <v>17.6</v>
       </c>
       <c r="Y15">
-        <v>90.3</v>
+        <v>86.5</v>
       </c>
       <c r="Z15">
-        <v>59.1</v>
+        <v>58.7</v>
       </c>
       <c r="AA15">
         <v>0.98</v>
@@ -8096,7 +8096,7 @@
         <v>82.90000000000001</v>
       </c>
       <c r="AM15">
-        <v>20.1</v>
+        <v>25.5</v>
       </c>
       <c r="AN15">
         <v>0.2</v>
@@ -8270,13 +8270,13 @@
         <v>52.7</v>
       </c>
       <c r="CS15">
-        <v>44.1</v>
+        <v>47.1</v>
       </c>
       <c r="CT15" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="CU15">
-        <v>2.2</v>
+        <v>10.2</v>
       </c>
       <c r="CV15" t="s">
         <v>159</v>
@@ -8323,10 +8323,10 @@
         <v>305</v>
       </c>
       <c r="J16">
-        <v>230.6</v>
+        <v>232.5</v>
       </c>
       <c r="K16">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="L16">
         <v>5</v>
@@ -8338,7 +8338,7 @@
         <v>0.67</v>
       </c>
       <c r="O16">
-        <v>25.07</v>
+        <v>20.57</v>
       </c>
       <c r="P16">
         <v>47.3</v>
@@ -8365,13 +8365,13 @@
         <v>0.6667</v>
       </c>
       <c r="X16">
-        <v>17.8</v>
+        <v>16.2</v>
       </c>
       <c r="Y16">
-        <v>90.3</v>
+        <v>86.59999999999999</v>
       </c>
       <c r="Z16">
-        <v>62.9</v>
+        <v>62.4</v>
       </c>
       <c r="AA16">
         <v>0.98</v>
@@ -8410,7 +8410,7 @@
         <v>99.90000000000001</v>
       </c>
       <c r="AM16">
-        <v>18.1</v>
+        <v>28.8</v>
       </c>
       <c r="AN16">
         <v>0.099</v>
@@ -8584,13 +8584,13 @@
         <v>56.7</v>
       </c>
       <c r="CS16">
-        <v>38.7</v>
+        <v>44.6</v>
       </c>
       <c r="CT16" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="CU16">
-        <v>3.1</v>
+        <v>11.1</v>
       </c>
       <c r="CV16" t="s">
         <v>159</v>
@@ -8637,10 +8637,10 @@
         <v>305</v>
       </c>
       <c r="J17">
-        <v>230.6</v>
+        <v>232.5</v>
       </c>
       <c r="K17">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="L17">
         <v>5</v>
@@ -8652,7 +8652,7 @@
         <v>1.31</v>
       </c>
       <c r="O17">
-        <v>19.47</v>
+        <v>14.03</v>
       </c>
       <c r="P17">
         <v>13.1</v>
@@ -8679,13 +8679,13 @@
         <v>0.6667</v>
       </c>
       <c r="X17">
-        <v>17.2</v>
+        <v>15.3</v>
       </c>
       <c r="Y17">
-        <v>89.7</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="Z17">
-        <v>57</v>
+        <v>57.1</v>
       </c>
       <c r="AA17">
         <v>0.98</v>
@@ -8724,7 +8724,7 @@
         <v>80</v>
       </c>
       <c r="AM17">
-        <v>16.1</v>
+        <v>21.9</v>
       </c>
       <c r="AN17">
         <v>0</v>
@@ -8898,7 +8898,7 @@
         <v>58.2</v>
       </c>
       <c r="CS17">
-        <v>14.1</v>
+        <v>17.3</v>
       </c>
       <c r="CT17" t="s">
         <v>159</v>
@@ -8951,7 +8951,7 @@
         <v>306</v>
       </c>
       <c r="J18">
-        <v>72.7</v>
+        <v>74.7</v>
       </c>
       <c r="K18">
         <v>0</v>
@@ -8966,7 +8966,7 @@
         <v>0.72</v>
       </c>
       <c r="O18">
-        <v>17.84</v>
+        <v>22.33</v>
       </c>
       <c r="P18">
         <v>4</v>
@@ -8993,13 +8993,13 @@
         <v>0.0833</v>
       </c>
       <c r="X18">
-        <v>16.1</v>
+        <v>17.7</v>
       </c>
       <c r="Y18">
-        <v>85.90000000000001</v>
+        <v>85.2</v>
       </c>
       <c r="Z18">
-        <v>64.7</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="AA18">
         <v>0.92</v>
@@ -9038,7 +9038,7 @@
         <v>28.3</v>
       </c>
       <c r="AM18">
-        <v>21.2</v>
+        <v>18.2</v>
       </c>
       <c r="AN18">
         <v>0.003</v>
@@ -9212,7 +9212,7 @@
         <v>60.4</v>
       </c>
       <c r="CS18">
-        <v>18.6</v>
+        <v>17</v>
       </c>
       <c r="CT18" t="s">
         <v>159</v>
@@ -9265,7 +9265,7 @@
         <v>306</v>
       </c>
       <c r="J19">
-        <v>72.7</v>
+        <v>74.7</v>
       </c>
       <c r="K19">
         <v>0.1</v>
@@ -9280,7 +9280,7 @@
         <v>0.26</v>
       </c>
       <c r="O19">
-        <v>13.15</v>
+        <v>16.1</v>
       </c>
       <c r="P19">
         <v>6.3</v>
@@ -9307,13 +9307,13 @@
         <v>0.0833</v>
       </c>
       <c r="X19">
-        <v>8.800000000000001</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="Y19">
-        <v>92.5</v>
+        <v>92</v>
       </c>
       <c r="Z19">
-        <v>64.90000000000001</v>
+        <v>64.8</v>
       </c>
       <c r="AA19">
         <v>0.92</v>
@@ -9352,7 +9352,7 @@
         <v>24</v>
       </c>
       <c r="AM19">
-        <v>14.3</v>
+        <v>12.2</v>
       </c>
       <c r="AN19">
         <v>0.002</v>
@@ -9526,7 +9526,7 @@
         <v>63.3</v>
       </c>
       <c r="CS19">
-        <v>14.1</v>
+        <v>13</v>
       </c>
       <c r="CT19" t="s">
         <v>159</v>
@@ -9579,7 +9579,7 @@
         <v>306</v>
       </c>
       <c r="J20">
-        <v>72.7</v>
+        <v>74.7</v>
       </c>
       <c r="K20">
         <v>1.1</v>
@@ -9594,7 +9594,7 @@
         <v>0.55</v>
       </c>
       <c r="O20">
-        <v>9.050000000000001</v>
+        <v>10.52</v>
       </c>
       <c r="P20">
         <v>4.3</v>
@@ -9621,13 +9621,13 @@
         <v>0.0833</v>
       </c>
       <c r="X20">
-        <v>7.7</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="Y20">
-        <v>94.8</v>
+        <v>94.59999999999999</v>
       </c>
       <c r="Z20">
-        <v>63.4</v>
+        <v>63.3</v>
       </c>
       <c r="AA20">
         <v>0.92</v>
@@ -9666,7 +9666,7 @@
         <v>18.7</v>
       </c>
       <c r="AM20">
-        <v>7</v>
+        <v>5.8</v>
       </c>
       <c r="AN20">
         <v>0</v>
@@ -9840,7 +9840,7 @@
         <v>67.2</v>
       </c>
       <c r="CS20">
-        <v>5.9</v>
+        <v>5.3</v>
       </c>
       <c r="CT20" t="s">
         <v>159</v>
@@ -9893,7 +9893,7 @@
         <v>306</v>
       </c>
       <c r="J21">
-        <v>72.7</v>
+        <v>74.7</v>
       </c>
       <c r="K21">
         <v>2.1</v>
@@ -9908,7 +9908,7 @@
         <v>0.66</v>
       </c>
       <c r="O21">
-        <v>3.51</v>
+        <v>4.5</v>
       </c>
       <c r="P21">
         <v>5.4</v>
@@ -9935,10 +9935,10 @@
         <v>0.0833</v>
       </c>
       <c r="X21">
-        <v>5.9</v>
+        <v>6.2</v>
       </c>
       <c r="Y21">
-        <v>95.7</v>
+        <v>95.5</v>
       </c>
       <c r="Z21">
         <v>59.4</v>
@@ -9980,7 +9980,7 @@
         <v>18.1</v>
       </c>
       <c r="AM21">
-        <v>2.7</v>
+        <v>1.8</v>
       </c>
       <c r="AN21">
         <v>0</v>
@@ -10154,7 +10154,7 @@
         <v>70.09999999999999</v>
       </c>
       <c r="CS21">
-        <v>2.3</v>
+        <v>1.8</v>
       </c>
       <c r="CT21" t="s">
         <v>159</v>
@@ -10207,7 +10207,7 @@
         <v>307</v>
       </c>
       <c r="J22">
-        <v>370.2</v>
+        <v>372.4</v>
       </c>
       <c r="K22">
         <v>0</v>
@@ -10222,7 +10222,7 @@
         <v>1.83</v>
       </c>
       <c r="O22">
-        <v>1.18</v>
+        <v>1.23</v>
       </c>
       <c r="P22">
         <v>7.4</v>
@@ -10521,10 +10521,10 @@
         <v>307</v>
       </c>
       <c r="J23">
-        <v>370.2</v>
+        <v>372.4</v>
       </c>
       <c r="K23">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="L23">
         <v>5</v>
@@ -10536,7 +10536,7 @@
         <v>1.43</v>
       </c>
       <c r="O23">
-        <v>2.62</v>
+        <v>0.75</v>
       </c>
       <c r="P23">
         <v>29.8</v>
@@ -10563,13 +10563,13 @@
         <v>0.1667</v>
       </c>
       <c r="X23">
-        <v>10.5</v>
+        <v>9.9</v>
       </c>
       <c r="Y23">
-        <v>94.7</v>
+        <v>95</v>
       </c>
       <c r="Z23">
-        <v>49.9</v>
+        <v>49.8</v>
       </c>
       <c r="AA23">
         <v>0.88</v>
@@ -10835,10 +10835,10 @@
         <v>307</v>
       </c>
       <c r="J24">
-        <v>370.2</v>
+        <v>372.4</v>
       </c>
       <c r="K24">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="L24">
         <v>5</v>
@@ -10850,7 +10850,7 @@
         <v>1.19</v>
       </c>
       <c r="O24">
-        <v>2.5</v>
+        <v>0.14</v>
       </c>
       <c r="P24">
         <v>0.8</v>
@@ -10877,10 +10877,10 @@
         <v>0.1667</v>
       </c>
       <c r="X24">
-        <v>9</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="Y24">
-        <v>93.40000000000001</v>
+        <v>93.8</v>
       </c>
       <c r="Z24">
         <v>50.4</v>
@@ -11149,10 +11149,10 @@
         <v>307</v>
       </c>
       <c r="J25">
-        <v>370.2</v>
+        <v>372.4</v>
       </c>
       <c r="K25">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="L25">
         <v>5</v>
@@ -11164,7 +11164,7 @@
         <v>1.09</v>
       </c>
       <c r="O25">
-        <v>1.58</v>
+        <v>1.3</v>
       </c>
       <c r="P25">
         <v>7.2</v>
@@ -11191,7 +11191,7 @@
         <v>0.1667</v>
       </c>
       <c r="X25">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
       <c r="Y25">
         <v>94</v>
@@ -11463,7 +11463,7 @@
         <v>308</v>
       </c>
       <c r="J26">
-        <v>195.3</v>
+        <v>197.5</v>
       </c>
       <c r="K26">
         <v>0</v>
@@ -11478,7 +11478,7 @@
         <v>1.74</v>
       </c>
       <c r="O26">
-        <v>0.84</v>
+        <v>0.65</v>
       </c>
       <c r="P26">
         <v>11.8</v>
@@ -11777,10 +11777,10 @@
         <v>308</v>
       </c>
       <c r="J27">
-        <v>195.3</v>
+        <v>197.5</v>
       </c>
       <c r="K27">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="L27">
         <v>5</v>
@@ -11792,7 +11792,7 @@
         <v>0.8</v>
       </c>
       <c r="O27">
-        <v>0.75</v>
+        <v>2.92</v>
       </c>
       <c r="P27">
         <v>6.6</v>
@@ -11819,10 +11819,10 @@
         <v>0.1667</v>
       </c>
       <c r="X27">
-        <v>11</v>
+        <v>11.7</v>
       </c>
       <c r="Y27">
-        <v>89.40000000000001</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="Z27">
         <v>46.4</v>
@@ -12044,7 +12044,7 @@
         <v>159</v>
       </c>
       <c r="CU27">
-        <v>10.3</v>
+        <v>10.2</v>
       </c>
       <c r="CV27" t="s">
         <v>159</v>
@@ -12091,10 +12091,10 @@
         <v>308</v>
       </c>
       <c r="J28">
-        <v>195.3</v>
+        <v>197.5</v>
       </c>
       <c r="K28">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="L28">
         <v>5</v>
@@ -12106,7 +12106,7 @@
         <v>0.54</v>
       </c>
       <c r="O28">
-        <v>2.09</v>
+        <v>5.78</v>
       </c>
       <c r="P28">
         <v>10.8</v>
@@ -12133,13 +12133,13 @@
         <v>0.1667</v>
       </c>
       <c r="X28">
-        <v>10.7</v>
+        <v>12</v>
       </c>
       <c r="Y28">
-        <v>88.09999999999999</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="Z28">
-        <v>48.2</v>
+        <v>48.3</v>
       </c>
       <c r="AA28">
         <v>0.9399999999999999</v>
@@ -12405,10 +12405,10 @@
         <v>308</v>
       </c>
       <c r="J29">
-        <v>195.3</v>
+        <v>197.5</v>
       </c>
       <c r="K29">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="L29">
         <v>5</v>
@@ -12420,7 +12420,7 @@
         <v>0.65</v>
       </c>
       <c r="O29">
-        <v>3.36</v>
+        <v>3.49</v>
       </c>
       <c r="P29">
         <v>40.8</v>
@@ -12672,7 +12672,7 @@
         <v>159</v>
       </c>
       <c r="CU29">
-        <v>16.3</v>
+        <v>16.2</v>
       </c>
       <c r="CV29" t="s">
         <v>159</v>
@@ -12719,7 +12719,7 @@
         <v>309</v>
       </c>
       <c r="J30">
-        <v>332.7</v>
+        <v>335</v>
       </c>
       <c r="K30">
         <v>0</v>
@@ -13033,10 +13033,10 @@
         <v>309</v>
       </c>
       <c r="J31">
-        <v>332.7</v>
+        <v>335</v>
       </c>
       <c r="K31">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="L31">
         <v>5</v>
@@ -13347,10 +13347,10 @@
         <v>309</v>
       </c>
       <c r="J32">
-        <v>332.7</v>
+        <v>335</v>
       </c>
       <c r="K32">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="L32">
         <v>5</v>
@@ -13661,10 +13661,10 @@
         <v>309</v>
       </c>
       <c r="J33">
-        <v>332.7</v>
+        <v>335</v>
       </c>
       <c r="K33">
-        <v>2.7</v>
+        <v>2.6</v>
       </c>
       <c r="L33">
         <v>5</v>
@@ -13975,7 +13975,7 @@
         <v>310</v>
       </c>
       <c r="J34">
-        <v>92.5</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="K34">
         <v>0</v>
@@ -13990,7 +13990,7 @@
         <v>1.3</v>
       </c>
       <c r="O34">
-        <v>0.82</v>
+        <v>7.18</v>
       </c>
       <c r="P34">
         <v>6.1</v>
@@ -14017,13 +14017,13 @@
         <v>0.6667</v>
       </c>
       <c r="X34">
-        <v>6.2</v>
+        <v>8.4</v>
       </c>
       <c r="Y34">
-        <v>92.90000000000001</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="Z34">
-        <v>70.90000000000001</v>
+        <v>70.7</v>
       </c>
       <c r="AA34">
         <v>1.02</v>
@@ -14062,7 +14062,7 @@
         <v>46.7</v>
       </c>
       <c r="AM34">
-        <v>5.6</v>
+        <v>8</v>
       </c>
       <c r="AN34">
         <v>0</v>
@@ -14236,7 +14236,7 @@
         <v>60.4</v>
       </c>
       <c r="CS34">
-        <v>3.5</v>
+        <v>4.9</v>
       </c>
       <c r="CT34" t="s">
         <v>159</v>
@@ -14289,10 +14289,10 @@
         <v>310</v>
       </c>
       <c r="J35">
-        <v>92.5</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="K35">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="L35">
         <v>5</v>
@@ -14304,7 +14304,7 @@
         <v>0.99</v>
       </c>
       <c r="O35">
-        <v>2.13</v>
+        <v>6.36</v>
       </c>
       <c r="P35">
         <v>3.5</v>
@@ -14331,13 +14331,13 @@
         <v>0.6667</v>
       </c>
       <c r="X35">
-        <v>3.9</v>
+        <v>5.3</v>
       </c>
       <c r="Y35">
-        <v>94.59999999999999</v>
+        <v>93.90000000000001</v>
       </c>
       <c r="Z35">
-        <v>70.7</v>
+        <v>70.5</v>
       </c>
       <c r="AA35">
         <v>1.02</v>
@@ -14376,7 +14376,7 @@
         <v>52.6</v>
       </c>
       <c r="AM35">
-        <v>7.2</v>
+        <v>9.5</v>
       </c>
       <c r="AN35">
         <v>0</v>
@@ -14550,7 +14550,7 @@
         <v>63.2</v>
       </c>
       <c r="CS35">
-        <v>5.3</v>
+        <v>6.6</v>
       </c>
       <c r="CT35" t="s">
         <v>159</v>
@@ -14603,10 +14603,10 @@
         <v>310</v>
       </c>
       <c r="J36">
-        <v>92.5</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="K36">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="L36">
         <v>5</v>
@@ -14618,7 +14618,7 @@
         <v>0.8100000000000001</v>
       </c>
       <c r="O36">
-        <v>5.34</v>
+        <v>5.02</v>
       </c>
       <c r="P36">
         <v>12.4</v>
@@ -14645,10 +14645,10 @@
         <v>0.6667</v>
       </c>
       <c r="X36">
-        <v>7.3</v>
+        <v>7.2</v>
       </c>
       <c r="Y36">
-        <v>91.59999999999999</v>
+        <v>91.7</v>
       </c>
       <c r="Z36">
         <v>61.6</v>
@@ -14917,10 +14917,10 @@
         <v>310</v>
       </c>
       <c r="J37">
-        <v>92.5</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="K37">
-        <v>2.7</v>
+        <v>2.6</v>
       </c>
       <c r="L37">
         <v>5</v>
@@ -14932,7 +14932,7 @@
         <v>1.26</v>
       </c>
       <c r="O37">
-        <v>7.17</v>
+        <v>6.47</v>
       </c>
       <c r="P37">
         <v>34.9</v>
@@ -14959,10 +14959,10 @@
         <v>0.6667</v>
       </c>
       <c r="X37">
-        <v>10.8</v>
+        <v>10.5</v>
       </c>
       <c r="Y37">
-        <v>84</v>
+        <v>84.2</v>
       </c>
       <c r="Z37">
         <v>60.7</v>
@@ -15231,10 +15231,10 @@
         <v>311</v>
       </c>
       <c r="J38">
-        <v>253.5</v>
+        <v>256</v>
       </c>
       <c r="K38">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L38">
         <v>5</v>
@@ -15545,10 +15545,10 @@
         <v>311</v>
       </c>
       <c r="J39">
-        <v>253.5</v>
+        <v>256</v>
       </c>
       <c r="K39">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="L39">
         <v>5</v>
@@ -15859,10 +15859,10 @@
         <v>311</v>
       </c>
       <c r="J40">
-        <v>253.5</v>
+        <v>256</v>
       </c>
       <c r="K40">
-        <v>2.1</v>
+        <v>2</v>
       </c>
       <c r="L40">
         <v>5</v>
@@ -16126,7 +16126,7 @@
         <v>159</v>
       </c>
       <c r="CU40">
-        <v>4</v>
+        <v>3.9</v>
       </c>
       <c r="CV40" t="s">
         <v>159</v>
@@ -16173,10 +16173,10 @@
         <v>311</v>
       </c>
       <c r="J41">
-        <v>253.5</v>
+        <v>256</v>
       </c>
       <c r="K41">
-        <v>3.1</v>
+        <v>3</v>
       </c>
       <c r="L41">
         <v>5</v>
@@ -16487,10 +16487,10 @@
         <v>312</v>
       </c>
       <c r="J42">
-        <v>313.4</v>
+        <v>315.9</v>
       </c>
       <c r="K42">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="L42">
         <v>5</v>
@@ -16502,7 +16502,7 @@
         <v>1.04</v>
       </c>
       <c r="O42">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="P42">
         <v>8.1</v>
@@ -16529,7 +16529,7 @@
         <v>0.6667</v>
       </c>
       <c r="X42">
-        <v>7.3</v>
+        <v>7.2</v>
       </c>
       <c r="Y42">
         <v>91.90000000000001</v>
@@ -16801,10 +16801,10 @@
         <v>312</v>
       </c>
       <c r="J43">
-        <v>313.4</v>
+        <v>315.9</v>
       </c>
       <c r="K43">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="L43">
         <v>5</v>
@@ -16816,7 +16816,7 @@
         <v>1.91</v>
       </c>
       <c r="O43">
-        <v>0.5</v>
+        <v>0.33</v>
       </c>
       <c r="P43">
         <v>26.7</v>
@@ -16843,7 +16843,7 @@
         <v>0.6667</v>
       </c>
       <c r="X43">
-        <v>11.2</v>
+        <v>11.1</v>
       </c>
       <c r="Y43">
         <v>90.5</v>
@@ -17115,10 +17115,10 @@
         <v>312</v>
       </c>
       <c r="J44">
-        <v>313.4</v>
+        <v>315.9</v>
       </c>
       <c r="K44">
-        <v>2.7</v>
+        <v>2.6</v>
       </c>
       <c r="L44">
         <v>5</v>
@@ -17429,10 +17429,10 @@
         <v>312</v>
       </c>
       <c r="J45">
-        <v>313.4</v>
+        <v>315.9</v>
       </c>
       <c r="K45">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="L45">
         <v>5</v>
@@ -17444,7 +17444,7 @@
         <v>1.31</v>
       </c>
       <c r="O45">
-        <v>0.5</v>
+        <v>0.17</v>
       </c>
       <c r="P45">
         <v>81.40000000000001</v>
@@ -17471,10 +17471,10 @@
         <v>0.6667</v>
       </c>
       <c r="X45">
-        <v>7.1</v>
+        <v>6.9</v>
       </c>
       <c r="Y45">
-        <v>92.2</v>
+        <v>92.3</v>
       </c>
       <c r="Z45">
         <v>73.7</v>
@@ -17516,7 +17516,7 @@
         <v>20.8</v>
       </c>
       <c r="AM45">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="AN45">
         <v>0</v>
@@ -17690,13 +17690,13 @@
         <v>65.8</v>
       </c>
       <c r="CS45">
-        <v>1.6</v>
+        <v>1.4</v>
       </c>
       <c r="CT45" t="s">
         <v>159</v>
       </c>
       <c r="CU45">
-        <v>8.4</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="CV45" t="s">
         <v>159</v>
@@ -17899,7 +17899,7 @@
         <v>110</v>
       </c>
       <c r="P3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="Q3">
         <v>5</v>
@@ -17925,7 +17925,7 @@
         <v>134</v>
       </c>
       <c r="G4">
-        <v>92.3</v>
+        <v>91.7</v>
       </c>
       <c r="H4">
         <v>8</v>
@@ -17934,7 +17934,7 @@
         <v>6</v>
       </c>
       <c r="J4">
-        <v>4</v>
+        <v>3.9</v>
       </c>
       <c r="K4">
         <v>2</v>
@@ -17978,7 +17978,7 @@
         <v>134</v>
       </c>
       <c r="G5">
-        <v>87.3</v>
+        <v>87</v>
       </c>
       <c r="H5">
         <v>8</v>
@@ -18005,7 +18005,7 @@
         <v>110</v>
       </c>
       <c r="P5" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="Q5">
         <v>5</v>
@@ -18031,7 +18031,7 @@
         <v>134</v>
       </c>
       <c r="G6">
-        <v>90.59999999999999</v>
+        <v>90.2</v>
       </c>
       <c r="H6">
         <v>7</v>
@@ -18040,7 +18040,7 @@
         <v>5</v>
       </c>
       <c r="J6">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="K6">
         <v>1</v>
@@ -18131,13 +18131,13 @@
         <v>102</v>
       </c>
       <c r="E8">
-        <v>57.4</v>
+        <v>57.3</v>
       </c>
       <c r="F8" t="s">
         <v>136</v>
       </c>
       <c r="G8">
-        <v>89</v>
+        <v>87.2</v>
       </c>
       <c r="H8">
         <v>5</v>
@@ -18164,7 +18164,7 @@
         <v>110</v>
       </c>
       <c r="P8" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="Q8">
         <v>5</v>
@@ -18243,7 +18243,7 @@
         <v>136</v>
       </c>
       <c r="G10">
-        <v>93</v>
+        <v>93.2</v>
       </c>
       <c r="H10">
         <v>2</v>
@@ -18296,7 +18296,7 @@
         <v>136</v>
       </c>
       <c r="G11">
-        <v>90.40000000000001</v>
+        <v>90.2</v>
       </c>
       <c r="H11">
         <v>1</v>
@@ -18376,7 +18376,7 @@
         <v>111</v>
       </c>
       <c r="P12" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="Q12">
         <v>5</v>

</xml_diff>